<commit_message>
temporary commit, before adding the conditional entropy
</commit_message>
<xml_diff>
--- a/apps_nicolo/multiIC_RPA_3species_5rxns_MAK_REINFORCE/dose_response_3species_5rxns_MAK_REINFORCE.xlsx
+++ b/apps_nicolo/multiIC_RPA_3species_5rxns_MAK_REINFORCE/dose_response_3species_5rxns_MAK_REINFORCE.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,11 @@
           <t>2025-11-20 15:49:46</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>2025-11-20 15:53:51</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +514,11 @@
           <t>https://www.comet.com/redsnic/dose-response-3species-5rxns-mak-reinforce/0f0a3b6ac9a14f8b86a5910dbb7054d8</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.comet.com/redsnic/dose-response-3species-5rxns-mak-reinforce/bccaed2c556c4193a425b54cb80a53c3</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -540,6 +550,9 @@
       <c r="I3" t="n">
         <v>5</v>
       </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -571,6 +584,9 @@
       <c r="I4" t="n">
         <v>3</v>
       </c>
+      <c r="J4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -602,6 +618,9 @@
       <c r="I5" t="n">
         <v>1</v>
       </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -633,6 +652,9 @@
       <c r="I6" t="n">
         <v>3840</v>
       </c>
+      <c r="J6" t="n">
+        <v>3840</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -664,6 +686,9 @@
       <c r="I7" t="b">
         <v>0</v>
       </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -695,6 +720,9 @@
       <c r="I8" t="n">
         <v>0.0001</v>
       </c>
+      <c r="J8" t="n">
+        <v>0.0001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -726,6 +754,9 @@
       <c r="I9" t="n">
         <v>300</v>
       </c>
+      <c r="J9" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -757,6 +788,9 @@
       <c r="I10" t="n">
         <v>5</v>
       </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -788,6 +822,9 @@
       <c r="I11" t="n">
         <v>1024</v>
       </c>
+      <c r="J11" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -819,6 +856,9 @@
       <c r="I12" t="n">
         <v>10240</v>
       </c>
+      <c r="J12" t="n">
+        <v>10240</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -850,6 +890,9 @@
       <c r="I13" t="n">
         <v>128</v>
       </c>
+      <c r="J13" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -897,6 +940,11 @@
           <t>{'entropy_weight': 0.01, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.01}</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>{'entropy_weight': 0.01, 'entropy_update_coefficient': 1, 'entropy_schedule': 1000, 'minimum_entropy_weight': 0.01}</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -944,6 +992,11 @@
           <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>{'risk': 0.95, 'risk_update': 0.0, 'max_risk': 1.0, 'risk_schedule': 1000}</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -975,6 +1028,9 @@
       <c r="I16" t="n">
         <v>1</v>
       </c>
+      <c r="J16" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1006,6 +1062,9 @@
       <c r="I17" t="n">
         <v>10</v>
       </c>
+      <c r="J17" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1037,6 +1096,9 @@
       <c r="I18" t="n">
         <v>100</v>
       </c>
+      <c r="J18" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1068,6 +1130,9 @@
       <c r="I19" t="n">
         <v>1000</v>
       </c>
+      <c r="J19" t="n">
+        <v>1000</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1099,6 +1164,9 @@
       <c r="I20" t="n">
         <v>2</v>
       </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1130,6 +1198,9 @@
       <c r="I21" t="n">
         <v>5</v>
       </c>
+      <c r="J21" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1173,6 +1244,11 @@
         </is>
       </c>
       <c r="I22" t="inlineStr">
+        <is>
+          <t>{'type': 'lognormal_1D'}</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>{'type': 'lognormal_1D'}</t>
         </is>

</xml_diff>